<commit_message>
Updated F16 constraints source file. Removed hardcoded values.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/Constraints.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/Constraints.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\Tasks\Spring_2026\MATLAB\Level_IV_Fidelity\Operator\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DEBEF0DA-17E6-43CA-B341-B4A0DBDCDD38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{189CA43C-D7CD-455E-AD9F-10EF66144209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="384" windowWidth="23256" windowHeight="12720" activeTab="1" xr2:uid="{A16C2A72-36AD-490A-A958-AABD199434F3}"/>
+    <workbookView xWindow="-120" yWindow="330" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{A16C2A72-36AD-490A-A958-AABD199434F3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,15 +40,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
   <si>
     <t>Altitude (ft)</t>
   </si>
   <si>
     <t>Max Mach</t>
-  </si>
-  <si>
-    <t>CD0</t>
   </si>
   <si>
     <t>Cruise</t>
@@ -81,18 +78,6 @@
     <t>W/Wto</t>
   </si>
   <si>
-    <t>K1</t>
-  </si>
-  <si>
-    <t>K2</t>
-  </si>
-  <si>
-    <t>alpha_dry</t>
-  </si>
-  <si>
-    <t>alpha_wet</t>
-  </si>
-  <si>
     <t>Combat Subsonic</t>
   </si>
   <si>
@@ -114,13 +99,7 @@
     <t>AB%</t>
   </si>
   <si>
-    <t>throttle lapse</t>
-  </si>
-  <si>
     <t>Distance (fT)</t>
-  </si>
-  <si>
-    <t>e</t>
   </si>
   <si>
     <t>CLmax</t>
@@ -888,66 +867,50 @@
   <sheetData>
     <row r="2" spans="3:25" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="3:25" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C5" s="1"/>
       <c r="D5" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>2</v>
+        <v>11</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J5" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="K5" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="K5" s="3" t="s">
+      <c r="L5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="N5" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="O5" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="P5" s="4" t="s">
-        <v>0</v>
-      </c>
-      <c r="Q5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="R5" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="S5" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="T5" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="U5" s="4" t="s">
-        <v>32</v>
-      </c>
+      <c r="M5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="N5" s="4"/>
+      <c r="O5" s="4"/>
+      <c r="P5" s="4"/>
+      <c r="Q5" s="4"/>
+      <c r="R5" s="4"/>
+      <c r="S5" s="4"/>
+      <c r="T5" s="4"/>
+      <c r="U5" s="4"/>
       <c r="V5" s="4"/>
       <c r="W5" s="4"/>
       <c r="X5" s="4"/>
@@ -960,43 +923,27 @@
       <c r="D6" s="6">
         <v>0.89966599999999997</v>
       </c>
-      <c r="E6" s="6">
-        <v>3.9316999999999998E-2</v>
-      </c>
-      <c r="F6" s="6">
-        <v>0.213727</v>
-      </c>
-      <c r="G6" s="6">
-        <v>0</v>
-      </c>
-      <c r="H6" s="6">
-        <v>0.29829299999999997</v>
-      </c>
-      <c r="I6" s="6">
-        <v>0.57698000000000005</v>
-      </c>
-      <c r="J6" s="7">
+      <c r="E6" s="7">
         <v>100</v>
       </c>
-      <c r="K6" s="7">
-        <v>0.57699999999999996</v>
-      </c>
-      <c r="L6" s="7">
-        <v>3.9316999999999998E-2</v>
-      </c>
-      <c r="M6" s="7">
-        <v>0.91400000000000003</v>
-      </c>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8">
+        <v>1</v>
+      </c>
+      <c r="H6" s="8">
+        <v>36000</v>
+      </c>
+      <c r="I6" s="8">
+        <v>1.6</v>
+      </c>
+      <c r="J6" s="8"/>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8"/>
+      <c r="M6" s="8"/>
       <c r="N6" s="8"/>
-      <c r="O6" s="8">
-        <v>1</v>
-      </c>
-      <c r="P6" s="8">
-        <v>36000</v>
-      </c>
-      <c r="Q6" s="8">
-        <v>1.6</v>
-      </c>
+      <c r="O6" s="8"/>
+      <c r="P6" s="8"/>
+      <c r="Q6" s="8"/>
       <c r="R6" s="8"/>
       <c r="S6" s="8"/>
       <c r="T6" s="8"/>
@@ -1008,48 +955,32 @@
     </row>
     <row r="7" spans="3:25" x14ac:dyDescent="0.25">
       <c r="C7" s="5" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="6">
         <v>0.89966599999999997</v>
       </c>
-      <c r="E7" s="6">
-        <v>1.6996000000000001E-2</v>
-      </c>
-      <c r="F7" s="10">
-        <v>0.116031</v>
-      </c>
-      <c r="G7" s="10">
-        <v>-6.3E-3</v>
-      </c>
-      <c r="H7" s="10">
-        <v>0.27111000000000002</v>
-      </c>
-      <c r="I7" s="10">
-        <v>0.33264199999999999</v>
-      </c>
-      <c r="J7" s="10">
+      <c r="E7" s="10">
         <v>0</v>
       </c>
-      <c r="K7" s="8">
-        <v>0.1711</v>
-      </c>
-      <c r="L7" s="8">
-        <v>1.6996000000000001E-2</v>
-      </c>
-      <c r="M7" s="7">
-        <v>0.91400000000000003</v>
-      </c>
+      <c r="F7" s="8"/>
+      <c r="G7" s="8">
+        <v>1</v>
+      </c>
+      <c r="H7" s="8">
+        <v>36000</v>
+      </c>
+      <c r="I7" s="8">
+        <v>0.87</v>
+      </c>
+      <c r="J7" s="8"/>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8"/>
+      <c r="M7" s="8"/>
       <c r="N7" s="8"/>
-      <c r="O7" s="8">
-        <v>1</v>
-      </c>
-      <c r="P7" s="8">
-        <v>36000</v>
-      </c>
-      <c r="Q7" s="8">
-        <v>0.87</v>
-      </c>
+      <c r="O7" s="8"/>
+      <c r="P7" s="8"/>
+      <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
       <c r="S7" s="8"/>
       <c r="T7" s="8"/>
@@ -1061,48 +992,32 @@
     </row>
     <row r="8" spans="3:25" x14ac:dyDescent="0.25">
       <c r="C8" s="9" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D8" s="6">
         <v>0.89966599999999997</v>
       </c>
-      <c r="E8" s="6">
-        <v>1.6996000000000001E-2</v>
-      </c>
-      <c r="F8" s="10">
-        <v>0.116031</v>
-      </c>
-      <c r="G8" s="10">
-        <v>-6.3E-3</v>
-      </c>
-      <c r="H8" s="10">
-        <v>0.138789</v>
-      </c>
-      <c r="I8" s="10">
-        <v>0.17029</v>
-      </c>
-      <c r="J8" s="10">
+      <c r="E8" s="10">
         <v>100</v>
       </c>
-      <c r="K8" s="8">
-        <v>0.17030000000000001</v>
-      </c>
-      <c r="L8" s="8">
-        <v>1.6996000000000001E-2</v>
-      </c>
-      <c r="M8" s="7">
-        <v>0.91400000000000003</v>
-      </c>
+      <c r="F8" s="8"/>
+      <c r="G8" s="8">
+        <v>1</v>
+      </c>
+      <c r="H8" s="8">
+        <v>50000</v>
+      </c>
+      <c r="I8" s="8">
+        <v>0.87</v>
+      </c>
+      <c r="J8" s="8"/>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8"/>
+      <c r="M8" s="8"/>
       <c r="N8" s="8"/>
-      <c r="O8" s="8">
-        <v>1</v>
-      </c>
-      <c r="P8" s="8">
-        <v>50000</v>
-      </c>
-      <c r="Q8" s="8">
-        <v>0.87</v>
-      </c>
+      <c r="O8" s="8"/>
+      <c r="P8" s="8"/>
+      <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
       <c r="S8" s="8"/>
       <c r="T8" s="8"/>
@@ -1114,48 +1029,32 @@
     </row>
     <row r="9" spans="3:25" ht="30" x14ac:dyDescent="0.25">
       <c r="C9" s="9" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="D9" s="6">
         <v>0.89966599999999997</v>
       </c>
-      <c r="E9" s="6">
-        <v>1.6996000000000001E-2</v>
-      </c>
-      <c r="F9" s="10">
-        <v>0.116031</v>
-      </c>
-      <c r="G9" s="10">
-        <v>-6.3E-3</v>
-      </c>
-      <c r="H9" s="10">
-        <v>0.55566199999999999</v>
+      <c r="E9" s="8">
+        <v>100</v>
+      </c>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="H9" s="8">
+        <v>20000</v>
       </c>
       <c r="I9" s="8">
-        <v>0.68177699999999997</v>
-      </c>
-      <c r="J9" s="8">
-        <v>100</v>
-      </c>
-      <c r="K9" s="8">
-        <v>0.68179999999999996</v>
-      </c>
-      <c r="L9" s="8">
-        <v>1.6996000000000001E-2</v>
-      </c>
-      <c r="M9" s="7">
-        <v>0.91400000000000003</v>
-      </c>
+        <v>0.87</v>
+      </c>
+      <c r="J9" s="8"/>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8"/>
+      <c r="M9" s="8"/>
       <c r="N9" s="8"/>
-      <c r="O9" s="8">
-        <v>4.5</v>
-      </c>
-      <c r="P9" s="8">
-        <v>20000</v>
-      </c>
-      <c r="Q9" s="8">
-        <v>0.87</v>
-      </c>
+      <c r="O9" s="8"/>
+      <c r="P9" s="8"/>
+      <c r="Q9" s="8"/>
       <c r="R9" s="8"/>
       <c r="S9" s="8"/>
       <c r="T9" s="8"/>
@@ -1167,48 +1066,32 @@
     </row>
     <row r="10" spans="3:25" ht="45" x14ac:dyDescent="0.25">
       <c r="C10" s="9" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="D10" s="6">
         <v>0.89966599999999997</v>
       </c>
-      <c r="E10" s="6">
-        <v>4.0613999999999997E-2</v>
-      </c>
-      <c r="F10" s="10">
-        <v>0.21940599999999999</v>
-      </c>
-      <c r="G10" s="10">
-        <v>-1E-3</v>
-      </c>
-      <c r="H10" s="10">
-        <v>0.35786200000000001</v>
+      <c r="E10" s="8">
+        <v>100</v>
+      </c>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="H10" s="8">
+        <v>36000</v>
       </c>
       <c r="I10" s="8">
-        <v>0.556558</v>
-      </c>
-      <c r="J10" s="8">
-        <v>100</v>
-      </c>
-      <c r="K10" s="8">
-        <v>0.55659999999999998</v>
-      </c>
-      <c r="L10" s="8">
-        <v>4.0613999999999997E-2</v>
-      </c>
-      <c r="M10" s="7">
-        <v>0.91400000000000003</v>
-      </c>
+        <v>1.4</v>
+      </c>
+      <c r="J10" s="8"/>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8"/>
+      <c r="M10" s="8"/>
       <c r="N10" s="8"/>
-      <c r="O10" s="8">
-        <v>1.4</v>
-      </c>
-      <c r="P10" s="8">
-        <v>36000</v>
-      </c>
-      <c r="Q10" s="8">
-        <v>1.4</v>
-      </c>
+      <c r="O10" s="8"/>
+      <c r="P10" s="8"/>
+      <c r="Q10" s="8"/>
       <c r="R10" s="8"/>
       <c r="S10" s="8"/>
       <c r="T10" s="8"/>
@@ -1220,54 +1103,38 @@
     </row>
     <row r="11" spans="3:25" ht="30" x14ac:dyDescent="0.25">
       <c r="C11" s="9" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="D11" s="6">
         <v>0.89966599999999997</v>
       </c>
-      <c r="E11" s="6">
-        <v>1.6996000000000001E-2</v>
-      </c>
-      <c r="F11" s="10">
-        <v>0.116031</v>
-      </c>
-      <c r="G11" s="10">
-        <v>-6.3E-3</v>
-      </c>
-      <c r="H11" s="10">
-        <v>0.70272699999999999</v>
+      <c r="E11" s="8">
+        <v>100</v>
+      </c>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8">
+        <v>1</v>
+      </c>
+      <c r="H11" s="8">
+        <v>10000</v>
       </c>
       <c r="I11" s="8">
-        <v>0.85355000000000003</v>
+        <v>0.87</v>
       </c>
       <c r="J11" s="8">
-        <v>100</v>
+        <v>500</v>
       </c>
       <c r="K11" s="8">
-        <v>0.85360000000000003</v>
-      </c>
-      <c r="L11" s="8">
-        <v>1.6996000000000001E-2</v>
-      </c>
-      <c r="M11" s="7">
-        <v>0.91400000000000003</v>
-      </c>
+        <v>1.2</v>
+      </c>
+      <c r="L11" s="8"/>
+      <c r="M11" s="8"/>
       <c r="N11" s="8"/>
-      <c r="O11" s="8">
-        <v>1</v>
-      </c>
-      <c r="P11" s="8">
-        <v>10000</v>
-      </c>
-      <c r="Q11" s="8">
-        <v>0.87</v>
-      </c>
-      <c r="R11" s="8">
-        <v>500</v>
-      </c>
-      <c r="S11" s="8">
-        <v>1.2</v>
-      </c>
+      <c r="O11" s="8"/>
+      <c r="P11" s="8"/>
+      <c r="Q11" s="8"/>
+      <c r="R11" s="8"/>
+      <c r="S11" s="8"/>
       <c r="T11" s="8"/>
       <c r="U11" s="8"/>
       <c r="V11" s="8"/>
@@ -1277,54 +1144,38 @@
     </row>
     <row r="12" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C12" s="11" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="D12" s="10">
         <v>1</v>
       </c>
-      <c r="E12" s="10">
-        <v>5.1996000000000001E-2</v>
-      </c>
-      <c r="F12" s="10">
-        <v>0.116031</v>
-      </c>
-      <c r="G12" s="10">
-        <v>-6.3E-3</v>
-      </c>
-      <c r="H12" s="10">
-        <v>0.939778</v>
-      </c>
-      <c r="I12" s="8">
-        <v>0.95505300000000004</v>
-      </c>
+      <c r="E12" s="10"/>
+      <c r="F12" s="8">
+        <v>1.2756700000000001</v>
+      </c>
+      <c r="G12" s="8"/>
+      <c r="H12" s="8">
+        <v>0</v>
+      </c>
+      <c r="I12" s="8"/>
       <c r="J12" s="8"/>
       <c r="K12" s="8">
-        <v>0.95505300000000004</v>
+        <v>1.3</v>
       </c>
       <c r="L12" s="8">
-        <v>5.1996000000000001E-2</v>
-      </c>
-      <c r="M12" s="7">
-        <v>0.91400000000000003</v>
-      </c>
-      <c r="N12" s="8">
-        <v>1.2756700000000001</v>
-      </c>
+        <v>4000</v>
+      </c>
+      <c r="M12" s="8">
+        <v>0.03</v>
+      </c>
+      <c r="N12" s="8"/>
       <c r="O12" s="8"/>
-      <c r="P12" s="8">
-        <v>0</v>
-      </c>
+      <c r="P12" s="8"/>
       <c r="Q12" s="8"/>
       <c r="R12" s="8"/>
-      <c r="S12" s="8">
-        <v>1.3</v>
-      </c>
-      <c r="T12" s="8">
-        <v>4000</v>
-      </c>
-      <c r="U12" s="8">
-        <v>0.03</v>
-      </c>
+      <c r="S12" s="8"/>
+      <c r="T12" s="8"/>
+      <c r="U12" s="8"/>
       <c r="V12" s="8"/>
       <c r="W12" s="8"/>
       <c r="X12" s="8"/>
@@ -1332,50 +1183,36 @@
     </row>
     <row r="13" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C13" s="11" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D13" s="10">
         <v>1</v>
       </c>
-      <c r="E13" s="10">
-        <v>5.1996000000000001E-2</v>
-      </c>
-      <c r="F13" s="10">
-        <v>0.116031</v>
-      </c>
-      <c r="G13" s="10">
-        <v>-6.3E-3</v>
-      </c>
-      <c r="H13" s="10">
-        <v>0.939778</v>
-      </c>
-      <c r="I13" s="8">
-        <v>0.95505300000000004</v>
-      </c>
+      <c r="E13" s="10"/>
+      <c r="F13" s="8">
+        <v>1.42591</v>
+      </c>
+      <c r="G13" s="8"/>
+      <c r="H13" s="8">
+        <v>0</v>
+      </c>
+      <c r="I13" s="8"/>
       <c r="J13" s="8"/>
       <c r="K13" s="8"/>
       <c r="L13" s="8">
-        <v>6.1996000000000002E-2</v>
-      </c>
-      <c r="M13" s="7">
-        <v>0.91400000000000003</v>
-      </c>
-      <c r="N13" s="8">
-        <v>1.42591</v>
-      </c>
+        <v>4000</v>
+      </c>
+      <c r="M13" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="N13" s="8"/>
       <c r="O13" s="8"/>
-      <c r="P13" s="8">
-        <v>0</v>
-      </c>
+      <c r="P13" s="8"/>
       <c r="Q13" s="8"/>
       <c r="R13" s="8"/>
       <c r="S13" s="8"/>
-      <c r="T13" s="8">
-        <v>4000</v>
-      </c>
-      <c r="U13" s="8">
-        <v>0.5</v>
-      </c>
+      <c r="T13" s="8"/>
+      <c r="U13" s="8"/>
       <c r="V13" s="8"/>
       <c r="W13" s="8"/>
       <c r="X13" s="8"/>
@@ -1782,7 +1619,7 @@
       <c r="Y29" s="8"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D6:Y29">
+  <conditionalFormatting sqref="D6:F11 D15:Y29 D12:E13 V6:Y14 D14:U14 F6:U13">
     <cfRule type="expression" dxfId="11" priority="1">
       <formula>ISNOTFORMULA(D6)</formula>
     </cfRule>
@@ -1807,7 +1644,7 @@
   <sheetData>
     <row r="2" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3" spans="3:15" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1816,19 +1653,19 @@
         <v>1</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>7</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>8</v>
       </c>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
@@ -1883,7 +1720,7 @@
     </row>
     <row r="6" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C6" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D6" s="10">
         <v>1.6</v>
@@ -1912,7 +1749,7 @@
     </row>
     <row r="7" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" s="10">
         <v>1</v>
@@ -1941,7 +1778,7 @@
     </row>
     <row r="8" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C8" s="9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D8" s="10">
         <v>100</v>
@@ -1985,7 +1822,7 @@
     </row>
     <row r="10" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C10" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D10" s="10"/>
       <c r="E10" s="10"/>
@@ -2283,25 +2120,25 @@
         <v>1</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I3" s="3" t="s">
-        <v>8</v>
-      </c>
       <c r="J3" s="3" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
@@ -2343,7 +2180,7 @@
     </row>
     <row r="5" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C5" s="9" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D5" s="10">
         <v>1.6</v>
@@ -2372,7 +2209,7 @@
     </row>
     <row r="6" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C6" s="9" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D6" s="10">
         <v>1</v>
@@ -2401,7 +2238,7 @@
     </row>
     <row r="7" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7" s="10">
         <v>100</v>
@@ -2445,7 +2282,7 @@
     </row>
     <row r="9" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C9" s="11" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
@@ -2464,7 +2301,7 @@
     </row>
     <row r="10" spans="3:15" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C10" s="11" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D10" s="10"/>
       <c r="E10" s="10"/>

</xml_diff>

<commit_message>
Constraint section works now. Produces optimal_WS and min_TW that disagree from Brandt.
</commit_message>
<xml_diff>
--- a/examples/F-16A B Block 10 and 15/Operator/Constraints.xlsx
+++ b/examples/F-16A B Block 10 and 15/Operator/Constraints.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\John Freeman\Desktop\Academics\VRMastersProgram\code\air-vehicle-design\examples\F-16A B Block 10 and 15\Operator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{189CA43C-D7CD-455E-AD9F-10EF66144209}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF5F724-2433-4F37-A7DC-F4DCB74AAF6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="330" windowWidth="29040" windowHeight="15990" activeTab="1" xr2:uid="{A16C2A72-36AD-490A-A958-AABD199434F3}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Constraints" sheetId="3" r:id="rId2"/>
-    <sheet name="Aero_Constraints" sheetId="2" r:id="rId3"/>
-    <sheet name="Requirements" sheetId="5" r:id="rId4"/>
-    <sheet name="Thrust_Constraints" sheetId="4" r:id="rId5"/>
+    <sheet name="OldConstraints" sheetId="6" r:id="rId3"/>
+    <sheet name="Aero_Constraints" sheetId="2" r:id="rId4"/>
+    <sheet name="Requirements" sheetId="5" r:id="rId5"/>
+    <sheet name="Thrust_Constraints" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,12 +41,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="33">
   <si>
     <t>Altitude (ft)</t>
   </si>
   <si>
     <t>Max Mach</t>
+  </si>
+  <si>
+    <t>CD0</t>
   </si>
   <si>
     <t>Cruise</t>
@@ -78,6 +82,18 @@
     <t>W/Wto</t>
   </si>
   <si>
+    <t>K1</t>
+  </si>
+  <si>
+    <t>K2</t>
+  </si>
+  <si>
+    <t>alpha_dry</t>
+  </si>
+  <si>
+    <t>alpha_wet</t>
+  </si>
+  <si>
     <t>Combat Subsonic</t>
   </si>
   <si>
@@ -99,7 +115,13 @@
     <t>AB%</t>
   </si>
   <si>
+    <t>throttle lapse</t>
+  </si>
+  <si>
     <t>Distance (fT)</t>
+  </si>
+  <si>
+    <t>e</t>
   </si>
   <si>
     <t>CLmax</t>
@@ -365,7 +387,28 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
+  <dxfs count="15">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="2"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -867,41 +910,41 @@
   <sheetData>
     <row r="2" spans="3:25" x14ac:dyDescent="0.25">
       <c r="D2" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="3:25" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C5" s="1"/>
       <c r="D5" s="2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H5" s="4" t="s">
         <v>0</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="J5" s="4" t="s">
-        <v>22</v>
+        <v>29</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="L5" s="4" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="M5" s="4" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="N5" s="4"/>
       <c r="O5" s="4"/>
@@ -955,7 +998,7 @@
     </row>
     <row r="7" spans="3:25" x14ac:dyDescent="0.25">
       <c r="C7" s="5" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" s="6">
         <v>0.89966599999999997</v>
@@ -992,7 +1035,7 @@
     </row>
     <row r="8" spans="3:25" x14ac:dyDescent="0.25">
       <c r="C8" s="9" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D8" s="6">
         <v>0.89966599999999997</v>
@@ -1029,7 +1072,7 @@
     </row>
     <row r="9" spans="3:25" ht="30" x14ac:dyDescent="0.25">
       <c r="C9" s="9" t="s">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="D9" s="6">
         <v>0.89966599999999997</v>
@@ -1066,7 +1109,7 @@
     </row>
     <row r="10" spans="3:25" ht="45" x14ac:dyDescent="0.25">
       <c r="C10" s="9" t="s">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D10" s="6">
         <v>0.89966599999999997</v>
@@ -1103,7 +1146,7 @@
     </row>
     <row r="11" spans="3:25" ht="30" x14ac:dyDescent="0.25">
       <c r="C11" s="9" t="s">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="D11" s="6">
         <v>0.89966599999999997</v>
@@ -1124,9 +1167,7 @@
       <c r="J11" s="8">
         <v>500</v>
       </c>
-      <c r="K11" s="8">
-        <v>1.2</v>
-      </c>
+      <c r="K11" s="8"/>
       <c r="L11" s="8"/>
       <c r="M11" s="8"/>
       <c r="N11" s="8"/>
@@ -1144,7 +1185,7 @@
     </row>
     <row r="12" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C12" s="11" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="D12" s="10">
         <v>1</v>
@@ -1153,14 +1194,14 @@
       <c r="F12" s="8">
         <v>1.2756700000000001</v>
       </c>
-      <c r="G12" s="8"/>
+      <c r="G12" s="10"/>
       <c r="H12" s="8">
         <v>0</v>
       </c>
       <c r="I12" s="8"/>
       <c r="J12" s="8"/>
       <c r="K12" s="8">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="L12" s="8">
         <v>4000</v>
@@ -1183,7 +1224,7 @@
     </row>
     <row r="13" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C13" s="11" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D13" s="10">
         <v>1</v>
@@ -1192,13 +1233,15 @@
       <c r="F13" s="8">
         <v>1.42591</v>
       </c>
-      <c r="G13" s="8"/>
+      <c r="G13" s="10"/>
       <c r="H13" s="8">
         <v>0</v>
       </c>
       <c r="I13" s="8"/>
       <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
+      <c r="K13" s="8">
+        <v>1.3</v>
+      </c>
       <c r="L13" s="8">
         <v>4000</v>
       </c>
@@ -1619,7 +1662,928 @@
       <c r="Y29" s="8"/>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D6:F11 D15:Y29 D12:E13 V6:Y14 D14:U14 F6:U13">
+  <conditionalFormatting sqref="D14:Y29 D12:E13 F6:F13 H6:H13 D6:I11 J6:Y10 J11:J12 L11:Y12 G12:M12 G13:Y13 K11">
+    <cfRule type="expression" dxfId="14" priority="1">
+      <formula>ISNOTFORMULA(D6)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="13" priority="2">
+      <formula>_xlfn.ISFORMULA(D6)</formula>
+    </cfRule>
+    <cfRule type="containsBlanks" dxfId="12" priority="3">
+      <formula>LEN(TRIM(D6))=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1259CA17-A39E-43E8-B1CD-AF71AEDA591C}">
+  <dimension ref="C2:Y29"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="7" width="11.28515625" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" customWidth="1"/>
+    <col min="9" max="9" width="9.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="3:25" x14ac:dyDescent="0.25">
+      <c r="D2" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="3:25" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C5" s="1"/>
+      <c r="D5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="O5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="P5" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="R5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="S5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="T5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="U5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="V5" s="4"/>
+      <c r="W5" s="4"/>
+      <c r="X5" s="4"/>
+      <c r="Y5" s="4"/>
+    </row>
+    <row r="6" spans="3:25" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C6" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" s="6">
+        <v>0.89966599999999997</v>
+      </c>
+      <c r="E6" s="6">
+        <v>3.9316999999999998E-2</v>
+      </c>
+      <c r="F6" s="6">
+        <v>0.213727</v>
+      </c>
+      <c r="G6" s="6">
+        <v>0</v>
+      </c>
+      <c r="H6" s="6">
+        <v>0.29829299999999997</v>
+      </c>
+      <c r="I6" s="6">
+        <v>0.57698000000000005</v>
+      </c>
+      <c r="J6" s="7">
+        <v>100</v>
+      </c>
+      <c r="K6" s="7">
+        <v>0.57699999999999996</v>
+      </c>
+      <c r="L6" s="7">
+        <v>3.9316999999999998E-2</v>
+      </c>
+      <c r="M6" s="7">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="N6" s="8"/>
+      <c r="O6" s="8">
+        <v>1</v>
+      </c>
+      <c r="P6" s="8">
+        <v>36000</v>
+      </c>
+      <c r="Q6" s="8">
+        <v>1.6</v>
+      </c>
+      <c r="R6" s="8"/>
+      <c r="S6" s="8"/>
+      <c r="T6" s="8"/>
+      <c r="U6" s="8"/>
+      <c r="V6" s="8"/>
+      <c r="W6" s="8"/>
+      <c r="X6" s="8"/>
+      <c r="Y6" s="8"/>
+    </row>
+    <row r="7" spans="3:25" x14ac:dyDescent="0.25">
+      <c r="C7" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="6">
+        <v>0.89966599999999997</v>
+      </c>
+      <c r="E7" s="6">
+        <v>1.6996000000000001E-2</v>
+      </c>
+      <c r="F7" s="10">
+        <v>0.116031</v>
+      </c>
+      <c r="G7" s="10">
+        <v>-6.3E-3</v>
+      </c>
+      <c r="H7" s="10">
+        <v>0.27111000000000002</v>
+      </c>
+      <c r="I7" s="10">
+        <v>0.33264199999999999</v>
+      </c>
+      <c r="J7" s="10">
+        <v>0</v>
+      </c>
+      <c r="K7" s="8">
+        <v>0.1711</v>
+      </c>
+      <c r="L7" s="8">
+        <v>1.6996000000000001E-2</v>
+      </c>
+      <c r="M7" s="7">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="N7" s="8"/>
+      <c r="O7" s="8">
+        <v>1</v>
+      </c>
+      <c r="P7" s="8">
+        <v>36000</v>
+      </c>
+      <c r="Q7" s="8">
+        <v>0.87</v>
+      </c>
+      <c r="R7" s="8"/>
+      <c r="S7" s="8"/>
+      <c r="T7" s="8"/>
+      <c r="U7" s="8"/>
+      <c r="V7" s="8"/>
+      <c r="W7" s="8"/>
+      <c r="X7" s="8"/>
+      <c r="Y7" s="8"/>
+    </row>
+    <row r="8" spans="3:25" x14ac:dyDescent="0.25">
+      <c r="C8" s="9" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="6">
+        <v>0.89966599999999997</v>
+      </c>
+      <c r="E8" s="6">
+        <v>1.6996000000000001E-2</v>
+      </c>
+      <c r="F8" s="10">
+        <v>0.116031</v>
+      </c>
+      <c r="G8" s="10">
+        <v>-6.3E-3</v>
+      </c>
+      <c r="H8" s="10">
+        <v>0.138789</v>
+      </c>
+      <c r="I8" s="10">
+        <v>0.17029</v>
+      </c>
+      <c r="J8" s="10">
+        <v>100</v>
+      </c>
+      <c r="K8" s="8">
+        <v>0.17030000000000001</v>
+      </c>
+      <c r="L8" s="8">
+        <v>1.6996000000000001E-2</v>
+      </c>
+      <c r="M8" s="7">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="N8" s="8"/>
+      <c r="O8" s="8">
+        <v>1</v>
+      </c>
+      <c r="P8" s="8">
+        <v>50000</v>
+      </c>
+      <c r="Q8" s="8">
+        <v>0.87</v>
+      </c>
+      <c r="R8" s="8"/>
+      <c r="S8" s="8"/>
+      <c r="T8" s="8"/>
+      <c r="U8" s="8"/>
+      <c r="V8" s="8"/>
+      <c r="W8" s="8"/>
+      <c r="X8" s="8"/>
+      <c r="Y8" s="8"/>
+    </row>
+    <row r="9" spans="3:25" ht="30" x14ac:dyDescent="0.25">
+      <c r="C9" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="6">
+        <v>0.89966599999999997</v>
+      </c>
+      <c r="E9" s="6">
+        <v>1.6996000000000001E-2</v>
+      </c>
+      <c r="F9" s="10">
+        <v>0.116031</v>
+      </c>
+      <c r="G9" s="10">
+        <v>-6.3E-3</v>
+      </c>
+      <c r="H9" s="10">
+        <v>0.55566199999999999</v>
+      </c>
+      <c r="I9" s="8">
+        <v>0.68177699999999997</v>
+      </c>
+      <c r="J9" s="8">
+        <v>100</v>
+      </c>
+      <c r="K9" s="8">
+        <v>0.68179999999999996</v>
+      </c>
+      <c r="L9" s="8">
+        <v>1.6996000000000001E-2</v>
+      </c>
+      <c r="M9" s="7">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="N9" s="8"/>
+      <c r="O9" s="8">
+        <v>4.5</v>
+      </c>
+      <c r="P9" s="8">
+        <v>20000</v>
+      </c>
+      <c r="Q9" s="8">
+        <v>0.87</v>
+      </c>
+      <c r="R9" s="8"/>
+      <c r="S9" s="8"/>
+      <c r="T9" s="8"/>
+      <c r="U9" s="8"/>
+      <c r="V9" s="8"/>
+      <c r="W9" s="8"/>
+      <c r="X9" s="8"/>
+      <c r="Y9" s="8"/>
+    </row>
+    <row r="10" spans="3:25" ht="45" x14ac:dyDescent="0.25">
+      <c r="C10" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="6">
+        <v>0.89966599999999997</v>
+      </c>
+      <c r="E10" s="6">
+        <v>4.0613999999999997E-2</v>
+      </c>
+      <c r="F10" s="10">
+        <v>0.21940599999999999</v>
+      </c>
+      <c r="G10" s="10">
+        <v>-1E-3</v>
+      </c>
+      <c r="H10" s="10">
+        <v>0.35786200000000001</v>
+      </c>
+      <c r="I10" s="8">
+        <v>0.556558</v>
+      </c>
+      <c r="J10" s="8">
+        <v>100</v>
+      </c>
+      <c r="K10" s="8">
+        <v>0.55659999999999998</v>
+      </c>
+      <c r="L10" s="8">
+        <v>4.0613999999999997E-2</v>
+      </c>
+      <c r="M10" s="7">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="N10" s="8"/>
+      <c r="O10" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="P10" s="8">
+        <v>36000</v>
+      </c>
+      <c r="Q10" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="R10" s="8"/>
+      <c r="S10" s="8"/>
+      <c r="T10" s="8"/>
+      <c r="U10" s="8"/>
+      <c r="V10" s="8"/>
+      <c r="W10" s="8"/>
+      <c r="X10" s="8"/>
+      <c r="Y10" s="8"/>
+    </row>
+    <row r="11" spans="3:25" ht="30" x14ac:dyDescent="0.25">
+      <c r="C11" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" s="6">
+        <v>0.89966599999999997</v>
+      </c>
+      <c r="E11" s="6">
+        <v>1.6996000000000001E-2</v>
+      </c>
+      <c r="F11" s="10">
+        <v>0.116031</v>
+      </c>
+      <c r="G11" s="10">
+        <v>-6.3E-3</v>
+      </c>
+      <c r="H11" s="10">
+        <v>0.70272699999999999</v>
+      </c>
+      <c r="I11" s="8">
+        <v>0.85355000000000003</v>
+      </c>
+      <c r="J11" s="8">
+        <v>100</v>
+      </c>
+      <c r="K11" s="8">
+        <v>0.85360000000000003</v>
+      </c>
+      <c r="L11" s="8">
+        <v>1.6996000000000001E-2</v>
+      </c>
+      <c r="M11" s="7">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="N11" s="8"/>
+      <c r="O11" s="8">
+        <v>1</v>
+      </c>
+      <c r="P11" s="8">
+        <v>10000</v>
+      </c>
+      <c r="Q11" s="8">
+        <v>0.87</v>
+      </c>
+      <c r="R11" s="8">
+        <v>500</v>
+      </c>
+      <c r="S11" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="T11" s="8"/>
+      <c r="U11" s="8"/>
+      <c r="V11" s="8"/>
+      <c r="W11" s="8"/>
+      <c r="X11" s="8"/>
+      <c r="Y11" s="8"/>
+    </row>
+    <row r="12" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C12" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="D12" s="10">
+        <v>1</v>
+      </c>
+      <c r="E12" s="10">
+        <v>5.1996000000000001E-2</v>
+      </c>
+      <c r="F12" s="10">
+        <v>0.116031</v>
+      </c>
+      <c r="G12" s="10">
+        <v>-6.3E-3</v>
+      </c>
+      <c r="H12" s="10">
+        <v>0.939778</v>
+      </c>
+      <c r="I12" s="8">
+        <v>0.95505300000000004</v>
+      </c>
+      <c r="J12" s="8"/>
+      <c r="K12" s="8">
+        <v>0.95505300000000004</v>
+      </c>
+      <c r="L12" s="8">
+        <v>5.1996000000000001E-2</v>
+      </c>
+      <c r="M12" s="7">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="N12" s="8">
+        <v>1.2756700000000001</v>
+      </c>
+      <c r="O12" s="8"/>
+      <c r="P12" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="8"/>
+      <c r="R12" s="8"/>
+      <c r="S12" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="T12" s="8">
+        <v>4000</v>
+      </c>
+      <c r="U12" s="8">
+        <v>0.03</v>
+      </c>
+      <c r="V12" s="8"/>
+      <c r="W12" s="8"/>
+      <c r="X12" s="8"/>
+      <c r="Y12" s="8"/>
+    </row>
+    <row r="13" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="10">
+        <v>1</v>
+      </c>
+      <c r="E13" s="10">
+        <v>5.1996000000000001E-2</v>
+      </c>
+      <c r="F13" s="10">
+        <v>0.116031</v>
+      </c>
+      <c r="G13" s="10">
+        <v>-6.3E-3</v>
+      </c>
+      <c r="H13" s="10">
+        <v>0.939778</v>
+      </c>
+      <c r="I13" s="8">
+        <v>0.95505300000000004</v>
+      </c>
+      <c r="J13" s="8"/>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8">
+        <v>6.1996000000000002E-2</v>
+      </c>
+      <c r="M13" s="7">
+        <v>0.91400000000000003</v>
+      </c>
+      <c r="N13" s="8">
+        <v>1.42591</v>
+      </c>
+      <c r="O13" s="8"/>
+      <c r="P13" s="8">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="8"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="8"/>
+      <c r="T13" s="8">
+        <v>4000</v>
+      </c>
+      <c r="U13" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="V13" s="8"/>
+      <c r="W13" s="8"/>
+      <c r="X13" s="8"/>
+      <c r="Y13" s="8"/>
+    </row>
+    <row r="14" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C14" s="11"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="8"/>
+      <c r="I14" s="8"/>
+      <c r="J14" s="8"/>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8"/>
+      <c r="M14" s="8"/>
+      <c r="N14" s="8"/>
+      <c r="O14" s="8"/>
+      <c r="P14" s="8"/>
+      <c r="Q14" s="8"/>
+      <c r="R14" s="8"/>
+      <c r="S14" s="8"/>
+      <c r="T14" s="8"/>
+      <c r="U14" s="8"/>
+      <c r="V14" s="8"/>
+      <c r="W14" s="8"/>
+      <c r="X14" s="8"/>
+      <c r="Y14" s="8"/>
+    </row>
+    <row r="15" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C15" s="11"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+      <c r="F15" s="10"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="8"/>
+      <c r="I15" s="8"/>
+      <c r="J15" s="8"/>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8"/>
+      <c r="M15" s="8"/>
+      <c r="N15" s="8"/>
+      <c r="O15" s="8"/>
+      <c r="P15" s="8"/>
+      <c r="Q15" s="8"/>
+      <c r="R15" s="8"/>
+      <c r="S15" s="8"/>
+      <c r="T15" s="8"/>
+      <c r="U15" s="8"/>
+      <c r="V15" s="8"/>
+      <c r="W15" s="8"/>
+      <c r="X15" s="8"/>
+      <c r="Y15" s="8"/>
+    </row>
+    <row r="16" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="11"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="8"/>
+      <c r="I16" s="8"/>
+      <c r="J16" s="8"/>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8"/>
+      <c r="M16" s="8"/>
+      <c r="N16" s="8"/>
+      <c r="O16" s="8"/>
+      <c r="P16" s="8"/>
+      <c r="Q16" s="8"/>
+      <c r="R16" s="8"/>
+      <c r="S16" s="8"/>
+      <c r="T16" s="8"/>
+      <c r="U16" s="8"/>
+      <c r="V16" s="8"/>
+      <c r="W16" s="8"/>
+      <c r="X16" s="8"/>
+      <c r="Y16" s="8"/>
+    </row>
+    <row r="17" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C17" s="11"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="10"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="8"/>
+      <c r="I17" s="8"/>
+      <c r="J17" s="8"/>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8"/>
+      <c r="M17" s="8"/>
+      <c r="N17" s="8"/>
+      <c r="O17" s="8"/>
+      <c r="P17" s="8"/>
+      <c r="Q17" s="8"/>
+      <c r="R17" s="8"/>
+      <c r="S17" s="8"/>
+      <c r="T17" s="8"/>
+      <c r="U17" s="8"/>
+      <c r="V17" s="8"/>
+      <c r="W17" s="8"/>
+      <c r="X17" s="8"/>
+      <c r="Y17" s="8"/>
+    </row>
+    <row r="18" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C18" s="11"/>
+      <c r="D18" s="10"/>
+      <c r="E18" s="10"/>
+      <c r="F18" s="10"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="8"/>
+      <c r="I18" s="8"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="8"/>
+      <c r="N18" s="8"/>
+      <c r="O18" s="8"/>
+      <c r="P18" s="8"/>
+      <c r="Q18" s="8"/>
+      <c r="R18" s="8"/>
+      <c r="S18" s="8"/>
+      <c r="T18" s="8"/>
+      <c r="U18" s="8"/>
+      <c r="V18" s="8"/>
+      <c r="W18" s="8"/>
+      <c r="X18" s="8"/>
+      <c r="Y18" s="8"/>
+    </row>
+    <row r="19" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C19" s="11"/>
+      <c r="D19" s="10"/>
+      <c r="E19" s="10"/>
+      <c r="F19" s="10"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="8"/>
+      <c r="I19" s="8"/>
+      <c r="J19" s="8"/>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8"/>
+      <c r="M19" s="8"/>
+      <c r="N19" s="8"/>
+      <c r="O19" s="8"/>
+      <c r="P19" s="8"/>
+      <c r="Q19" s="8"/>
+      <c r="R19" s="8"/>
+      <c r="S19" s="8"/>
+      <c r="T19" s="8"/>
+      <c r="U19" s="8"/>
+      <c r="V19" s="8"/>
+      <c r="W19" s="8"/>
+      <c r="X19" s="8"/>
+      <c r="Y19" s="8"/>
+    </row>
+    <row r="20" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C20" s="11"/>
+      <c r="D20" s="10"/>
+      <c r="E20" s="10"/>
+      <c r="F20" s="10"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="8"/>
+      <c r="I20" s="8"/>
+      <c r="J20" s="8"/>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="8"/>
+      <c r="N20" s="8"/>
+      <c r="O20" s="8"/>
+      <c r="P20" s="8"/>
+      <c r="Q20" s="8"/>
+      <c r="R20" s="8"/>
+      <c r="S20" s="8"/>
+      <c r="T20" s="8"/>
+      <c r="U20" s="8"/>
+      <c r="V20" s="8"/>
+      <c r="W20" s="8"/>
+      <c r="X20" s="8"/>
+      <c r="Y20" s="8"/>
+    </row>
+    <row r="21" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C21" s="11"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="10"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="8"/>
+      <c r="I21" s="8"/>
+      <c r="J21" s="8"/>
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="8"/>
+      <c r="N21" s="8"/>
+      <c r="O21" s="8"/>
+      <c r="P21" s="8"/>
+      <c r="Q21" s="8"/>
+      <c r="R21" s="8"/>
+      <c r="S21" s="8"/>
+      <c r="T21" s="8"/>
+      <c r="U21" s="8"/>
+      <c r="V21" s="8"/>
+      <c r="W21" s="8"/>
+      <c r="X21" s="8"/>
+      <c r="Y21" s="8"/>
+    </row>
+    <row r="22" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C22" s="11"/>
+      <c r="D22" s="10"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
+      <c r="H22" s="8"/>
+      <c r="I22" s="8"/>
+      <c r="J22" s="8"/>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8"/>
+      <c r="M22" s="8"/>
+      <c r="N22" s="8"/>
+      <c r="O22" s="8"/>
+      <c r="P22" s="8"/>
+      <c r="Q22" s="8"/>
+      <c r="R22" s="8"/>
+      <c r="S22" s="8"/>
+      <c r="T22" s="8"/>
+      <c r="U22" s="8"/>
+      <c r="V22" s="8"/>
+      <c r="W22" s="8"/>
+      <c r="X22" s="8"/>
+      <c r="Y22" s="8"/>
+    </row>
+    <row r="23" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C23" s="11"/>
+      <c r="D23" s="10"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
+      <c r="H23" s="8"/>
+      <c r="I23" s="8"/>
+      <c r="J23" s="8"/>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="8"/>
+      <c r="N23" s="8"/>
+      <c r="O23" s="8"/>
+      <c r="P23" s="8"/>
+      <c r="Q23" s="8"/>
+      <c r="R23" s="8"/>
+      <c r="S23" s="8"/>
+      <c r="T23" s="8"/>
+      <c r="U23" s="8"/>
+      <c r="V23" s="8"/>
+      <c r="W23" s="8"/>
+      <c r="X23" s="8"/>
+      <c r="Y23" s="8"/>
+    </row>
+    <row r="24" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C24" s="11"/>
+      <c r="D24" s="10"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
+      <c r="H24" s="8"/>
+      <c r="I24" s="8"/>
+      <c r="J24" s="8"/>
+      <c r="K24" s="8"/>
+      <c r="L24" s="8"/>
+      <c r="M24" s="8"/>
+      <c r="N24" s="8"/>
+      <c r="O24" s="8"/>
+      <c r="P24" s="8"/>
+      <c r="Q24" s="8"/>
+      <c r="R24" s="8"/>
+      <c r="S24" s="8"/>
+      <c r="T24" s="8"/>
+      <c r="U24" s="8"/>
+      <c r="V24" s="8"/>
+      <c r="W24" s="8"/>
+      <c r="X24" s="8"/>
+      <c r="Y24" s="8"/>
+    </row>
+    <row r="25" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C25" s="11"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
+      <c r="H25" s="8"/>
+      <c r="I25" s="8"/>
+      <c r="J25" s="8"/>
+      <c r="K25" s="8"/>
+      <c r="L25" s="8"/>
+      <c r="M25" s="8"/>
+      <c r="N25" s="8"/>
+      <c r="O25" s="8"/>
+      <c r="P25" s="8"/>
+      <c r="Q25" s="8"/>
+      <c r="R25" s="8"/>
+      <c r="S25" s="8"/>
+      <c r="T25" s="8"/>
+      <c r="U25" s="8"/>
+      <c r="V25" s="8"/>
+      <c r="W25" s="8"/>
+      <c r="X25" s="8"/>
+      <c r="Y25" s="8"/>
+    </row>
+    <row r="26" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C26" s="11"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
+      <c r="H26" s="8"/>
+      <c r="I26" s="8"/>
+      <c r="J26" s="8"/>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8"/>
+      <c r="M26" s="8"/>
+      <c r="N26" s="8"/>
+      <c r="O26" s="8"/>
+      <c r="P26" s="8"/>
+      <c r="Q26" s="8"/>
+      <c r="R26" s="8"/>
+      <c r="S26" s="8"/>
+      <c r="T26" s="8"/>
+      <c r="U26" s="8"/>
+      <c r="V26" s="8"/>
+      <c r="W26" s="8"/>
+      <c r="X26" s="8"/>
+      <c r="Y26" s="8"/>
+    </row>
+    <row r="27" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C27" s="11"/>
+      <c r="D27" s="10"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
+      <c r="H27" s="8"/>
+      <c r="I27" s="8"/>
+      <c r="J27" s="8"/>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8"/>
+      <c r="M27" s="8"/>
+      <c r="N27" s="8"/>
+      <c r="O27" s="8"/>
+      <c r="P27" s="8"/>
+      <c r="Q27" s="8"/>
+      <c r="R27" s="8"/>
+      <c r="S27" s="8"/>
+      <c r="T27" s="8"/>
+      <c r="U27" s="8"/>
+      <c r="V27" s="8"/>
+      <c r="W27" s="8"/>
+      <c r="X27" s="8"/>
+      <c r="Y27" s="8"/>
+    </row>
+    <row r="28" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C28" s="11"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
+      <c r="H28" s="8"/>
+      <c r="I28" s="8"/>
+      <c r="J28" s="8"/>
+      <c r="K28" s="8"/>
+      <c r="L28" s="8"/>
+      <c r="M28" s="8"/>
+      <c r="N28" s="8"/>
+      <c r="O28" s="8"/>
+      <c r="P28" s="8"/>
+      <c r="Q28" s="8"/>
+      <c r="R28" s="8"/>
+      <c r="S28" s="8"/>
+      <c r="T28" s="8"/>
+      <c r="U28" s="8"/>
+      <c r="V28" s="8"/>
+      <c r="W28" s="8"/>
+      <c r="X28" s="8"/>
+      <c r="Y28" s="8"/>
+    </row>
+    <row r="29" spans="3:25" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C29" s="11"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
+      <c r="H29" s="8"/>
+      <c r="I29" s="8"/>
+      <c r="J29" s="8"/>
+      <c r="K29" s="8"/>
+      <c r="L29" s="8"/>
+      <c r="M29" s="8"/>
+      <c r="N29" s="8"/>
+      <c r="O29" s="8"/>
+      <c r="P29" s="8"/>
+      <c r="Q29" s="8"/>
+      <c r="R29" s="8"/>
+      <c r="S29" s="8"/>
+      <c r="T29" s="8"/>
+      <c r="U29" s="8"/>
+      <c r="V29" s="8"/>
+      <c r="W29" s="8"/>
+      <c r="X29" s="8"/>
+      <c r="Y29" s="8"/>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="D6:Y29">
     <cfRule type="expression" dxfId="11" priority="1">
       <formula>ISNOTFORMULA(D6)</formula>
     </cfRule>
@@ -1634,7 +2598,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A5B8E17F-F93C-4259-85CC-A015389E4C4E}">
   <dimension ref="C2:O27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1644,7 +2608,7 @@
   <sheetData>
     <row r="2" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="D2" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="3:15" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1653,19 +2617,19 @@
         <v>1</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
@@ -1720,7 +2684,7 @@
     </row>
     <row r="6" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C6" s="9" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D6" s="10">
         <v>1.6</v>
@@ -1749,7 +2713,7 @@
     </row>
     <row r="7" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D7" s="10">
         <v>1</v>
@@ -1778,7 +2742,7 @@
     </row>
     <row r="8" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C8" s="9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D8" s="10">
         <v>100</v>
@@ -1822,7 +2786,7 @@
     </row>
     <row r="10" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C10" s="11" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D10" s="10"/>
       <c r="E10" s="10"/>
@@ -2108,7 +3072,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1A10F3C-9DF3-4A3B-A79B-116DE712CC4A}">
   <dimension ref="C2:O27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2120,25 +3084,25 @@
         <v>1</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
@@ -2180,7 +3144,7 @@
     </row>
     <row r="5" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C5" s="9" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" s="10">
         <v>1.6</v>
@@ -2209,7 +3173,7 @@
     </row>
     <row r="6" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C6" s="9" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="10">
         <v>1</v>
@@ -2238,7 +3202,7 @@
     </row>
     <row r="7" spans="3:15" x14ac:dyDescent="0.25">
       <c r="C7" s="9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D7" s="10">
         <v>100</v>
@@ -2282,7 +3246,7 @@
     </row>
     <row r="9" spans="3:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C9" s="11" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
@@ -2301,7 +3265,7 @@
     </row>
     <row r="10" spans="3:15" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C10" s="11" t="s">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="D10" s="10"/>
       <c r="E10" s="10"/>
@@ -2591,7 +3555,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6367FCC9-8212-4D1B-890F-B035FF9196ED}">
   <dimension ref="B1:N26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>

</xml_diff>